<commit_message>
Save first 20 of 50 full-text omics screens in batch B005
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/omics_screening/omics_screening_cumulative.xlsx
+++ b/results/ad-oxygen-literature-20261006/omics_screening/omics_screening_cumulative.xlsx
@@ -19,9 +19,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'筛查总表'!$A$1:$AF$427</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'目标测序研究'!$A$1:$AF$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'数据项目与样本'!$A$1:$W$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'证据记录'!$A$1:$L$158</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'待确认与相关线索'!$A$1:$P$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'批次进度与统计'!$A$1:$D$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'证据记录'!$A$1:$L$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'待确认与相关线索'!$A$1:$P$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'批次进度与统计'!$A$1:$D$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'口径与字段说明'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12029,22 +12029,58 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
-      <c r="M88" s="2" t="inlineStr"/>
-      <c r="N88" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；水质、光谱/GC、Microtox及动力学</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O88" s="2" t="inlineStr"/>
-      <c r="P88" s="2" t="inlineStr"/>
-      <c r="Q88" s="2" t="inlineStr"/>
-      <c r="R88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>Direct Black22染料/乙醇合成废水</t>
+        </is>
+      </c>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>0.25±0.05 L/min；连续或30 min/2 h间歇</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr">
+        <is>
+          <t>R1严格厌氧；R2厌氧12 h+微曝气11 h；R3间歇微曝气</t>
+        </is>
+      </c>
       <c r="S88" s="2" t="inlineStr"/>
       <c r="T88" s="2" t="inlineStr"/>
       <c r="U88" s="2" t="inlineStr"/>
-      <c r="V88" s="2" t="inlineStr"/>
-      <c r="W88" s="2" t="inlineStr"/>
+      <c r="V88" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.4（PDF2–3页）为配水、SBR运行、水质/染料光谱、GC、Microtox毒性和动力学；sequencing batch reactor是序批式反应器术语，不是测序。未报告核酸建库或目标组学。</t>
+        </is>
+      </c>
+      <c r="W88" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–10页定位；方法PDF2–3页§2.1–2.4</t>
+        </is>
+      </c>
       <c r="X88" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04646/fulltext/fulltext__published__e1d4e0f3c97d519f.pdf"]</t>
@@ -12068,13 +12104,21 @@
       <c r="AB88" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC88" s="2" t="inlineStr"/>
+      <c r="AC88" s="2" t="inlineStr">
+        <is>
+          <t>正文提及SI用于NMR纯度和动力学计算；当前无独立原件，保留缺口，不追下载。</t>
+        </is>
+      </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE88" s="2" t="inlineStr"/>
+          <t>["R04646-E01", "R04646-E02"]</t>
+        </is>
+      </c>
+      <c r="AE88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:08:59.157148+00:00</t>
+        </is>
+      </c>
       <c r="AF88" s="2" t="inlineStr"/>
     </row>
     <row r="89" ht="60" customHeight="1">
@@ -12121,22 +12165,58 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr"/>
-      <c r="M89" s="2" t="inlineStr"/>
-      <c r="N89" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；AMPTS/BMP、GC、粒径及SMA</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O89" s="2" t="inlineStr"/>
-      <c r="P89" s="2" t="inlineStr"/>
-      <c r="Q89" s="2" t="inlineStr"/>
-      <c r="R89" s="2" t="inlineStr"/>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>合成市政废水；纤维素对照</t>
+        </is>
+      </c>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>3/5 bar微气泡白水处理接种污泥</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr">
+        <is>
+          <t>0/3/5 bar污泥；空白与纤维素对照；另有SMA实验</t>
+        </is>
+      </c>
       <c r="S89" s="2" t="inlineStr"/>
       <c r="T89" s="2" t="inlineStr"/>
       <c r="U89" s="2" t="inlineStr"/>
-      <c r="V89" s="2" t="inlineStr"/>
-      <c r="W89" s="2" t="inlineStr"/>
+      <c r="V89" s="2" t="inlineStr">
+        <is>
+          <t>51页学位研究；完整第3章（PDF14–23页）为底物、接种、加压白水、AMPTS和GC产气、粒径与SMA；附录I–IV为TS/VS、粒径仪截图及AMPTS/SMA数值表，无目标测序。低文字页已查看原页缩略图，均为封面、装置照片、粒径或产气表。</t>
+        </is>
+      </c>
+      <c r="W89" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–51页定位；第3章PDF14–23页完整；附录PDF38–51页；低文字PDF1/23/39–48/51视觉核查</t>
+        </is>
+      </c>
       <c r="X89" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04700/fulltext/fulltext__thesis__40ac0de29f75851c.pdf"]</t>
@@ -12160,13 +12240,21 @@
       <c r="AB89" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC89" s="2" t="inlineStr"/>
+      <c r="AC89" s="2" t="inlineStr">
+        <is>
+          <t>无独立SI；论文内附录I–IV已检查，非测序材料。</t>
+        </is>
+      </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE89" s="2" t="inlineStr"/>
+          <t>["R04700-E01", "R04700-E02"]</t>
+        </is>
+      </c>
+      <c r="AE89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:09:50.240337+00:00</t>
+        </is>
+      </c>
       <c r="AF89" s="2" t="inlineStr"/>
     </row>
     <row r="90" ht="60" customHeight="1">
@@ -12321,22 +12409,58 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr"/>
-      <c r="M91" s="2" t="inlineStr"/>
-      <c r="N91" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>细菌/古菌16S扩增子MiSeq（非目标）</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O91" s="2" t="inlineStr"/>
-      <c r="P91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>初沉污泥60%+剩余污泥40%</t>
+        </is>
+      </c>
       <c r="Q91" s="2" t="inlineStr"/>
       <c r="R91" s="2" t="inlineStr"/>
-      <c r="S91" s="2" t="inlineStr"/>
-      <c r="T91" s="2" t="inlineStr"/>
+      <c r="S91" s="2" t="inlineStr">
+        <is>
+          <t>Illumina MiSeq（16S扩增子）</t>
+        </is>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
+          <t>MA及Raw各1份污泥，共2份</t>
+        </is>
+      </c>
       <c r="U91" s="2" t="inlineStr"/>
-      <c r="V91" s="2" t="inlineStr"/>
-      <c r="W91" s="2" t="inlineStr"/>
+      <c r="V91" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.5（PDF2–3页）已读：总DNA后细菌338F/806R和古菌Arch524F/958R扩增16S，纯化amplicons后MiSeq、97% OTU。酶活为ELISA；无shotgun或群落RNA测序。</t>
+        </is>
+      </c>
+      <c r="W91" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–9页定位；方法PDF2–3页§2</t>
+        </is>
+      </c>
       <c r="X91" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04786/fulltext/fulltext__published__ea18005b6cd10f40.pdf"]</t>
@@ -12360,13 +12484,21 @@
       <c r="AB91" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC91" s="2" t="inlineStr"/>
+      <c r="AC91" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE91" s="2" t="inlineStr"/>
+          <t>["R04786-E01"]</t>
+        </is>
+      </c>
+      <c r="AE91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:09:50.268655+00:00</t>
+        </is>
+      </c>
       <c r="AF91" s="2" t="inlineStr"/>
     </row>
     <row r="92" ht="60" customHeight="1">
@@ -12417,22 +12549,58 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr"/>
-      <c r="M92" s="2" t="inlineStr"/>
-      <c r="N92" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；农场脱硫监测及经济分析</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O92" s="2" t="inlineStr"/>
-      <c r="P92" s="2" t="inlineStr"/>
-      <c r="Q92" s="2" t="inlineStr"/>
-      <c r="R92" s="2" t="inlineStr"/>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>奶牛粪与食物废物共消化</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>农场2顶空空气2.86 m3/h</t>
+        </is>
+      </c>
+      <c r="R92" s="2" t="inlineStr">
+        <is>
+          <t>农场1氧化铁/钢丝绒吸附；农场2生物微曝气脱硫</t>
+        </is>
+      </c>
       <c r="S92" s="2" t="inlineStr"/>
       <c r="T92" s="2" t="inlineStr"/>
       <c r="U92" s="2" t="inlineStr"/>
-      <c r="V92" s="2" t="inlineStr"/>
-      <c r="W92" s="2" t="inlineStr"/>
+      <c r="V92" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.4（PDF3–4页）为两厂装置、气体连续监测、维护成本、脱硫计算及统计；无核酸、建库、测序或组学复用。</t>
+        </is>
+      </c>
+      <c r="W92" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–13页定位；方法PDF3–4页§2</t>
+        </is>
+      </c>
       <c r="X92" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04796/fulltext/fulltext__published__6844f12fe56c174d.pdf"]</t>
@@ -12456,13 +12624,21 @@
       <c r="AB92" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC92" s="2" t="inlineStr"/>
+      <c r="AC92" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE92" s="2" t="inlineStr"/>
+          <t>["R04796-E01"]</t>
+        </is>
+      </c>
+      <c r="AE92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:09:50.299325+00:00</t>
+        </is>
+      </c>
       <c r="AF92" s="2" t="inlineStr"/>
     </row>
     <row r="93" ht="60" customHeight="1">
@@ -12513,22 +12689,58 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr"/>
-      <c r="M93" s="2" t="inlineStr"/>
-      <c r="N93" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>PCR-DGGE群落指纹（非目标）</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O93" s="2" t="inlineStr"/>
-      <c r="P93" s="2" t="inlineStr"/>
-      <c r="Q93" s="2" t="inlineStr"/>
-      <c r="R93" s="2" t="inlineStr"/>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>乙醇合成废水及400 mg/L硫酸钠</t>
+        </is>
+      </c>
+      <c r="Q93" s="2" t="inlineStr">
+        <is>
+          <t>0.1/0.3 mL/min；泥床内、泥床上方或顶空</t>
+        </is>
+      </c>
+      <c r="R93" s="2" t="inlineStr">
+        <is>
+          <t>R1先厌氧再泥床上微曝气；R2顶空/泥床微曝气</t>
+        </is>
+      </c>
       <c r="S93" s="2" t="inlineStr"/>
       <c r="T93" s="2" t="inlineStr"/>
       <c r="U93" s="2" t="inlineStr"/>
-      <c r="V93" s="2" t="inlineStr"/>
-      <c r="W93" s="2" t="inlineStr"/>
+      <c r="V93" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1、2.3–2.6（PDF5–6页）为反应器、曝气策略、标准水质、PCR-DGGE及生态指数。无目标测序；PDF23低文字原页为DGGE胶图，PDF17为利益声明，已视觉核查。</t>
+        </is>
+      </c>
+      <c r="W93" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–27页定位；方法PDF5–6页§2；PDF21图注及23胶图；低文字PDF17/23原页核查</t>
+        </is>
+      </c>
       <c r="X93" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04803/fulltext/fulltext__published__3e98d6cf0fefd5e7.pdf"]</t>
@@ -12552,13 +12764,21 @@
       <c r="AB93" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC93" s="2" t="inlineStr"/>
+      <c r="AC93" s="2" t="inlineStr">
+        <is>
+          <t>无独立SI；接受稿后部图表属于正文，DGGE胶图已核查。</t>
+        </is>
+      </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE93" s="2" t="inlineStr"/>
+          <t>["R04803-E01"]</t>
+        </is>
+      </c>
+      <c r="AE93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:09:50.328543+00:00</t>
+        </is>
+      </c>
       <c r="AF93" s="2" t="inlineStr"/>
     </row>
     <row r="94" ht="60" customHeight="1">
@@ -12713,22 +12933,58 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr"/>
-      <c r="M95" s="2" t="inlineStr"/>
-      <c r="N95" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；厌氧培养菌落计数及理化/GC</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O95" s="2" t="inlineStr"/>
-      <c r="P95" s="2" t="inlineStr"/>
-      <c r="Q95" s="2" t="inlineStr"/>
-      <c r="R95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>棕榈油厂废水POME</t>
+        </is>
+      </c>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t>产酸段每日注入相当工作液5%的空气，产甲烷段不曝气</t>
+        </is>
+      </c>
+      <c r="R95" s="2" t="inlineStr">
+        <is>
+          <t>牛粪与生物柴油废水来源接种物；产酸pH4/5</t>
+        </is>
+      </c>
       <c r="S95" s="2" t="inlineStr"/>
       <c r="T95" s="2" t="inlineStr"/>
       <c r="U95" s="2" t="inlineStr"/>
-      <c r="V95" s="2" t="inlineStr"/>
-      <c r="W95" s="2" t="inlineStr"/>
+      <c r="V95" s="2" t="inlineStr">
+        <is>
+          <t>完整RESEARCH METHODOLOGY（PDF2–4页）包括材料、两段AD、sCOD/VFA/GC与厌氧总菌落计数CFU；未报告DNA/RNA提取、建库或测序。</t>
+        </is>
+      </c>
+      <c r="W95" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–8页定位；方法PDF2–4页</t>
+        </is>
+      </c>
       <c r="X95" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04889/fulltext/fulltext__published__860a0532503787f8.pdf"]</t>
@@ -12752,13 +13008,21 @@
       <c r="AB95" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC95" s="2" t="inlineStr"/>
+      <c r="AC95" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE95" s="2" t="inlineStr"/>
+          <t>["R04889-E01", "R04889-E02"]</t>
+        </is>
+      </c>
+      <c r="AE95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:11:20.392454+00:00</t>
+        </is>
+      </c>
       <c r="AF95" s="2" t="inlineStr"/>
     </row>
     <row r="96" ht="60" customHeight="1">
@@ -12809,22 +13073,66 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr"/>
-      <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA及mcrA扩增子HiSeq（非目标）；宏转录组仅未来建议</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O96" s="2" t="inlineStr"/>
-      <c r="P96" s="2" t="inlineStr"/>
-      <c r="Q96" s="2" t="inlineStr"/>
-      <c r="R96" s="2" t="inlineStr"/>
-      <c r="S96" s="2" t="inlineStr"/>
-      <c r="T96" s="2" t="inlineStr"/>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>Napier草</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>ORP控制间歇O2，1 mL/min，隔日开关</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr">
+        <is>
+          <t>三次重复实验中厌氧与微曝气，ORP基线+25 mV</t>
+        </is>
+      </c>
+      <c r="S96" s="2" t="inlineStr">
+        <is>
+          <t>Illumina HiSeq2000（16S及mcrA靶基因）</t>
+        </is>
+      </c>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>三次重复各两时点，6份主分析样本；文中12个BioSample编号对应两个标记数据，未核实逐编号映射</t>
+        </is>
+      </c>
       <c r="U96" s="2" t="inlineStr"/>
-      <c r="V96" s="2" t="inlineStr"/>
-      <c r="W96" s="2" t="inlineStr"/>
+      <c r="V96" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.6（PDF2–3页）明确515F/806R扩增16S和mcrA3F/mcrA3R扩增mcrA后HiSeq、mothur/OTU；宏转录组在讨论为未来所需分析。DOCX补充方法为ORP、化学和热力学，不含额外shotgun/RNA建库。</t>
+        </is>
+      </c>
+      <c r="W96" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–10页定位；方法PDF2–3页§2；PDF7–8页宏转录组建议；DOCX全部588段落/表格</t>
+        </is>
+      </c>
       <c r="X96" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04899/fulltext/fulltext__published__92f0b2f1ad01522c.pdf"]</t>
@@ -12848,13 +13156,21 @@
       <c r="AB96" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC96" s="2" t="inlineStr"/>
+      <c r="AC96" s="2" t="inlineStr">
+        <is>
+          <t>题名/作者核实DOCX已读；补充ORP/化学/热力学，Table S2为扩增子OTU丰度，其余运行/理化表图，无目标测序。</t>
+        </is>
+      </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE96" s="2" t="inlineStr"/>
+          <t>["R04899-E01", "R04899-E02", "R04899-E03", "R04899-E04"]</t>
+        </is>
+      </c>
+      <c r="AE96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:11:20.426341+00:00</t>
+        </is>
+      </c>
       <c r="AF96" s="2" t="inlineStr"/>
     </row>
     <row r="97" ht="60" customHeight="1">
@@ -12905,22 +13221,58 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K97" s="2" t="inlineStr"/>
-      <c r="L97" s="2" t="inlineStr"/>
-      <c r="M97" s="2" t="inlineStr"/>
-      <c r="N97" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；发酵产气与动力学模型</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O97" s="2" t="inlineStr"/>
-      <c r="P97" s="2" t="inlineStr"/>
-      <c r="Q97" s="2" t="inlineStr"/>
-      <c r="R97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>模拟餐厨废物和污泥</t>
+        </is>
+      </c>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>空气0/5/10/15/20 mL组</t>
+        </is>
+      </c>
+      <c r="R97" s="2" t="inlineStr">
+        <is>
+          <t>五组厌氧/微曝气发酵，37°C、50天</t>
+        </is>
+      </c>
       <c r="S97" s="2" t="inlineStr"/>
       <c r="T97" s="2" t="inlineStr"/>
       <c r="U97" s="2" t="inlineStr"/>
-      <c r="V97" s="2" t="inlineStr"/>
-      <c r="W97" s="2" t="inlineStr"/>
+      <c r="V97" s="2" t="inlineStr">
+        <is>
+          <t>完整Materials and methods及Model establishment（PDF2–6页）为模拟食物废物批次发酵、每日产气、Logistic/Gompertz/一阶模型拟合，无核酸、测序或组学复用。</t>
+        </is>
+      </c>
+      <c r="W97" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–13页定位；实验方法PDF2–3页；模型PDF3–6页</t>
+        </is>
+      </c>
       <c r="X97" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04912/fulltext/fulltext__published__ba09ba8854601318.pdf"]</t>
@@ -12944,13 +13296,21 @@
       <c r="AB97" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC97" s="2" t="inlineStr"/>
+      <c r="AC97" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE97" s="2" t="inlineStr"/>
+          <t>["R04912-E01"]</t>
+        </is>
+      </c>
+      <c r="AE97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:11:20.456203+00:00</t>
+        </is>
+      </c>
       <c r="AF97" s="2" t="inlineStr"/>
     </row>
     <row r="98" ht="60" customHeight="1">
@@ -13001,22 +13361,58 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；全规模脱硫运行监测</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O98" s="2" t="inlineStr"/>
-      <c r="P98" s="2" t="inlineStr"/>
-      <c r="Q98" s="2" t="inlineStr"/>
-      <c r="R98" s="2" t="inlineStr"/>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>高固体污泥90%与食物废物相关物10%共消化</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>三消化罐顶空空气，剩余O2设定0.2–2.0%</t>
+        </is>
+      </c>
+      <c r="R98" s="2" t="inlineStr">
+        <is>
+          <t>三台55°C全规模消化罐81周不同供氧阶段</t>
+        </is>
+      </c>
       <c r="S98" s="2" t="inlineStr"/>
       <c r="T98" s="2" t="inlineStr"/>
       <c r="U98" s="2" t="inlineStr"/>
-      <c r="V98" s="2" t="inlineStr"/>
-      <c r="W98" s="2" t="inlineStr"/>
+      <c r="V98" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.3（PDF2页）为厂站、运行条件、气体流量/组分、固体/氨氮/碱度；未报告核酸或测序。</t>
+        </is>
+      </c>
+      <c r="W98" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–6页定位；方法PDF2页§2</t>
+        </is>
+      </c>
       <c r="X98" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04922/fulltext/fulltext__published__d4f609c42961a5d2.pdf"]</t>
@@ -13040,13 +13436,21 @@
       <c r="AB98" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC98" s="2" t="inlineStr"/>
+      <c r="AC98" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE98" s="2" t="inlineStr"/>
+          <t>["R04922-E01"]</t>
+        </is>
+      </c>
+      <c r="AE98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:11:20.485837+00:00</t>
+        </is>
+      </c>
       <c r="AF98" s="2" t="inlineStr"/>
     </row>
     <row r="99" ht="60" customHeight="1">
@@ -13097,22 +13501,58 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr"/>
-      <c r="M99" s="2" t="inlineStr"/>
-      <c r="N99" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；UASB运行、VS/VFA和产气模型</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O99" s="2" t="inlineStr"/>
-      <c r="P99" s="2" t="inlineStr"/>
-      <c r="Q99" s="2" t="inlineStr"/>
-      <c r="R99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>酒糟废水vinasse，牛粪接种</t>
+        </is>
+      </c>
+      <c r="Q99" s="2" t="inlineStr">
+        <is>
+          <t>每日取样后注气；DI无气/DII低气/DIII高气</t>
+        </is>
+      </c>
+      <c r="R99" s="2" t="inlineStr">
+        <is>
+          <t>三档空气投加及一阶降解模型</t>
+        </is>
+      </c>
       <c r="S99" s="2" t="inlineStr"/>
       <c r="T99" s="2" t="inlineStr"/>
       <c r="U99" s="2" t="inlineStr"/>
-      <c r="V99" s="2" t="inlineStr"/>
-      <c r="W99" s="2" t="inlineStr"/>
+      <c r="V99" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.2（PDF4–5页）为接种活化、UASB再循环、VS/VFA/排水量气；其余定量产酸模型，不含DNA/RNA建库或测序。</t>
+        </is>
+      </c>
+      <c r="W99" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–10页定位；方法PDF4–5页§2</t>
+        </is>
+      </c>
       <c r="X99" s="2" t="inlineStr">
         <is>
           <t>["original_files/R04928/fulltext/fulltext__published__9d47028c02204ac0.pdf"]</t>
@@ -13136,13 +13576,21 @@
       <c r="AB99" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC99" s="2" t="inlineStr"/>
+      <c r="AC99" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE99" s="2" t="inlineStr"/>
+          <t>["R04928-E01"]</t>
+        </is>
+      </c>
+      <c r="AE99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:11:20.514509+00:00</t>
+        </is>
+      </c>
       <c r="AF99" s="2" t="inlineStr"/>
     </row>
     <row r="100" ht="60" customHeight="1">
@@ -13293,22 +13741,58 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K101" s="2" t="inlineStr"/>
-      <c r="L101" s="2" t="inlineStr"/>
-      <c r="M101" s="2" t="inlineStr"/>
-      <c r="N101" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>16S V3–V4扩增子MiSeq（非目标）</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O101" s="2" t="inlineStr"/>
-      <c r="P101" s="2" t="inlineStr"/>
-      <c r="Q101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>2-丁烯醛生产废水</t>
+        </is>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>回流出水曝气，DO0.2–0.5 mg/L</t>
+        </is>
+      </c>
       <c r="R101" s="2" t="inlineStr"/>
-      <c r="S101" s="2" t="inlineStr"/>
+      <c r="S101" s="2" t="inlineStr">
+        <is>
+          <t>Illumina MiSeq</t>
+        </is>
+      </c>
       <c r="T101" s="2" t="inlineStr"/>
       <c r="U101" s="2" t="inlineStr"/>
-      <c r="V101" s="2" t="inlineStr"/>
-      <c r="W101" s="2" t="inlineStr"/>
+      <c r="V101" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.6（PDF2–3页）：EPS/核酸含量比色、EEM/PARAFAC及16S V3–V4 340F/805R扩增子测序；核酸定量不等同宏基因组。DOCX为装置/PCA、GCMS化合物表和16S多样性表，无额外目标流程。</t>
+        </is>
+      </c>
+      <c r="W101" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–9页定位；方法PDF2–3页；DOCX全部349段落及表S1/S2</t>
+        </is>
+      </c>
       <c r="X101" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05065/fulltext/fulltext__published__239adeaf9a5df55a.pdf"]</t>
@@ -13332,13 +13816,21 @@
       <c r="AB101" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC101" s="2" t="inlineStr"/>
+      <c r="AC101" s="2" t="inlineStr">
+        <is>
+          <t>题名/作者匹配DOCX全部文本和表格已读；无目标测序或编号。</t>
+        </is>
+      </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE101" s="2" t="inlineStr"/>
+          <t>["R05065-E01", "R05065-E02"]</t>
+        </is>
+      </c>
+      <c r="AE101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:12:59.723435+00:00</t>
+        </is>
+      </c>
       <c r="AF101" s="2" t="inlineStr"/>
     </row>
     <row r="102" ht="60" customHeight="1">
@@ -13493,22 +13985,62 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K103" s="2" t="inlineStr"/>
-      <c r="L103" s="2" t="inlineStr"/>
-      <c r="M103" s="2" t="inlineStr"/>
-      <c r="N103" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA扩增子HiSeq（非目标）</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O103" s="2" t="inlineStr"/>
-      <c r="P103" s="2" t="inlineStr"/>
-      <c r="Q103" s="2" t="inlineStr"/>
-      <c r="R103" s="2" t="inlineStr"/>
-      <c r="S103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>葡萄糖/三溴苯酚TBP合成废水</t>
+        </is>
+      </c>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>回流曝气；DO0.11/0.68/1.51 mg/L等阶段</t>
+        </is>
+      </c>
+      <c r="R103" s="2" t="inlineStr">
+        <is>
+          <t>R1活性污泥；R2加磁铁矿</t>
+        </is>
+      </c>
+      <c r="S103" s="2" t="inlineStr">
+        <is>
+          <t>Illumina HiSeq（16S）</t>
+        </is>
+      </c>
       <c r="T103" s="2" t="inlineStr"/>
       <c r="U103" s="2" t="inlineStr"/>
-      <c r="V103" s="2" t="inlineStr"/>
-      <c r="W103" s="2" t="inlineStr"/>
+      <c r="V103" s="2" t="inlineStr">
+        <is>
+          <t>完整Materials and Methods（PDF2–3页）：物化/酶活/显微及明确16S 515F/806R PCR、HiSeq、97% OTU/QIIME。DOCX仅种泥理化表及COD/稀释曲线/铁效应图，无额外目标测序。</t>
+        </is>
+      </c>
+      <c r="W103" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–9页定位；方法PDF2–3页；DOCX全部63段落</t>
+        </is>
+      </c>
       <c r="X103" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05173/fulltext/fulltext__published__dedf2d646e952ba0.pdf"]</t>
@@ -13532,13 +14064,21 @@
       <c r="AB103" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AC103" s="2" t="inlineStr"/>
+      <c r="AC103" s="2" t="inlineStr">
+        <is>
+          <t>DOCX缺独立题名/DOI，目录内容相符但保留唯一归属待核实；无可归属目标编号。</t>
+        </is>
+      </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE103" s="2" t="inlineStr"/>
+          <t>["R05173-E01", "R05173-E02", "R05173-E03"]</t>
+        </is>
+      </c>
+      <c r="AE103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:12:59.757033+00:00</t>
+        </is>
+      </c>
       <c r="AF103" s="2" t="inlineStr"/>
     </row>
     <row r="104" ht="60" customHeight="1">
@@ -13693,22 +14233,58 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K105" s="2" t="inlineStr"/>
-      <c r="L105" s="2" t="inlineStr"/>
-      <c r="M105" s="2" t="inlineStr"/>
-      <c r="N105" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；LPMO酶制剂、GC与HPAEC/NMR</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O105" s="2" t="inlineStr"/>
-      <c r="P105" s="2" t="inlineStr"/>
-      <c r="Q105" s="2" t="inlineStr"/>
-      <c r="R105" s="2" t="inlineStr"/>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>Avicel、云杉/桦木及富木质素残渣</t>
+        </is>
+      </c>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>厌氧/空气顶空及H2O2补加比较</t>
+        </is>
+      </c>
+      <c r="R105" s="2" t="inlineStr">
+        <is>
+          <t>酶/煮沸酶、NcLPMO9C、Celluclast及无酶/接种物对照</t>
+        </is>
+      </c>
       <c r="S105" s="2" t="inlineStr"/>
       <c r="T105" s="2" t="inlineStr"/>
       <c r="U105" s="2" t="inlineStr"/>
-      <c r="V105" s="2" t="inlineStr"/>
-      <c r="W105" s="2" t="inlineStr"/>
+      <c r="V105" s="2" t="inlineStr">
+        <is>
+          <t>完整Methods（PDF10–12页）为底物/成分、酶制剂、接种物、产气GC和氧化产物HPAEC；NcLPMO9C表达纯化非群落RNA测序。现有DOCX为色谱/甲烷曲线。PDF13泛指additional data可索取，但无目标测序，不计相关reads可索取候选。</t>
+        </is>
+      </c>
+      <c r="W105" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–14页定位；Methods PDF10–12页；数据声明PDF13页；DOCX全部72段落</t>
+        </is>
+      </c>
       <c r="X105" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05213/fulltext/fulltext__published__bcab84a15ce93062.pdf"]</t>
@@ -13732,13 +14308,21 @@
       <c r="AB105" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC105" s="2" t="inlineStr"/>
+      <c r="AC105" s="2" t="inlineStr">
+        <is>
+          <t>官方历史关联DOCX题名作者相符；全部图注为色谱与产气。</t>
+        </is>
+      </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE105" s="2" t="inlineStr"/>
+          <t>["R05213-E01", "R05213-E02", "R05213-E03", "R05213-E04"]</t>
+        </is>
+      </c>
+      <c r="AE105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:12:59.794409+00:00</t>
+        </is>
+      </c>
       <c r="AF105" s="2" t="inlineStr"/>
     </row>
     <row r="106" ht="60" customHeight="1">
@@ -13789,22 +14373,66 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K106" s="2" t="inlineStr"/>
-      <c r="L106" s="2" t="inlineStr"/>
-      <c r="M106" s="2" t="inlineStr"/>
-      <c r="N106" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>细菌/古菌16S扩增子MiSeq（非目标）</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O106" s="2" t="inlineStr"/>
-      <c r="P106" s="2" t="inlineStr"/>
-      <c r="Q106" s="2" t="inlineStr"/>
-      <c r="R106" s="2" t="inlineStr"/>
-      <c r="S106" s="2" t="inlineStr"/>
-      <c r="T106" s="2" t="inlineStr"/>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>鸡粪</t>
+        </is>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>1.4/2.8/4.2 mL O2/gVS，顶空载体连续/脉冲供气</t>
+        </is>
+      </c>
+      <c r="R106" s="2" t="inlineStr">
+        <is>
+          <t>R1厌氧；R2分四供气阶段，顶空尼龙载体</t>
+        </is>
+      </c>
+      <c r="S106" s="2" t="inlineStr">
+        <is>
+          <t>Illumina MiSeq（16S）</t>
+        </is>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>第120天R1/R2液相及R2载体；每类两份采样</t>
+        </is>
+      </c>
       <c r="U106" s="2" t="inlineStr"/>
-      <c r="V106" s="2" t="inlineStr"/>
-      <c r="W106" s="2" t="inlineStr"/>
+      <c r="V106" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.5（PDF2–4页）：化学/统计及338F/806R细菌、524F/958R古菌16S PCR、MiSeq、97% OTU。metagenome只出现在末页参考文献，不是本研究方法。</t>
+        </is>
+      </c>
+      <c r="W106" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–10页定位；方法PDF2–4页§2；参考文献PDF10页</t>
+        </is>
+      </c>
       <c r="X106" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05319/fulltext/fulltext__published__865dcb7f90757119.pdf"]</t>
@@ -13828,13 +14456,21 @@
       <c r="AB106" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC106" s="2" t="inlineStr"/>
+      <c r="AC106" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE106" s="2" t="inlineStr"/>
+          <t>["R05319-E01", "R05319-E02"]</t>
+        </is>
+      </c>
+      <c r="AE106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:13:19.954706+00:00</t>
+        </is>
+      </c>
       <c r="AF106" s="2" t="inlineStr"/>
     </row>
     <row r="107" ht="60" customHeight="1">
@@ -13885,22 +14521,62 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K107" s="2" t="inlineStr"/>
-      <c r="L107" s="2" t="inlineStr"/>
-      <c r="M107" s="2" t="inlineStr"/>
-      <c r="N107" s="2" t="inlineStr"/>
-      <c r="O107" s="2" t="inlineStr"/>
-      <c r="P107" s="2" t="inlineStr"/>
-      <c r="Q107" s="2" t="inlineStr"/>
-      <c r="R107" s="2" t="inlineStr"/>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>待确认：菌群组成已报告但测序方法未说明</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>未说明；仅报告细菌门/真菌纲，不能确认是否目标测序</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>7 证据不足，待确认</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>正文§2.1报告16个细菌门和7个真菌纲，但完整§2.1–2.6未交代核酸提取、靶标/引物、建库/测序或数据来源。现有匹配题名DOCX只有显微、FTIR和XRD图，无法区分扩增子、目标组学或既有分析。不能仅按菌群分类层级判断阴性。</t>
+        </is>
+      </c>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>油菜秸秆及两相消化水解产酸发酵液</t>
+        </is>
+      </c>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>0/20/60/120 mL O2/gVS/d，预处理10天</t>
+        </is>
+      </c>
+      <c r="R107" s="2" t="inlineStr">
+        <is>
+          <t>发酵液、灭菌过滤液和去离子水对照</t>
+        </is>
+      </c>
       <c r="S107" s="2" t="inlineStr"/>
       <c r="T107" s="2" t="inlineStr"/>
       <c r="U107" s="2" t="inlineStr"/>
-      <c r="V107" s="2" t="inlineStr"/>
-      <c r="W107" s="2" t="inlineStr"/>
+      <c r="V107" s="2" t="inlineStr">
+        <is>
+          <t>已完整阅读§2.1–2.6（PDF2–3页）及现有DOCX，主体为生物预处理、理化/GC/SEM/FTIR/XRD。预处理液菌群组成的分析来源和类型不明，保留待确认；全文及附件未定位编号或相关测序数据声明。</t>
+        </is>
+      </c>
+      <c r="W107" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–7页定位；方法PDF2–3页§2；DOCX全部22段落</t>
+        </is>
+      </c>
       <c r="X107" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05396/fulltext/fulltext__published__0a746b3ef69be3a5.pdf"]</t>
@@ -13924,14 +14600,22 @@
       <c r="AB107" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC107" s="2" t="inlineStr"/>
+      <c r="AC107" s="2" t="inlineStr">
+        <is>
+          <t>题名/作者核实DOCX仅菌丝/SEM/FTIR/XRD图，未补充菌群方法/编号。</t>
+        </is>
+      </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["R05396-E01", "R05396-E02"]</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr"/>
-      <c r="AF107" s="2" t="inlineStr"/>
+      <c r="AF107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:13:19.987967+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="60" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -13981,22 +14665,58 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K108" s="2" t="inlineStr"/>
-      <c r="L108" s="2" t="inlineStr"/>
-      <c r="M108" s="2" t="inlineStr"/>
-      <c r="N108" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；菌培养/显微/Gram染色及工程分析</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O108" s="2" t="inlineStr"/>
-      <c r="P108" s="2" t="inlineStr"/>
-      <c r="Q108" s="2" t="inlineStr"/>
-      <c r="R108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>猪粪沼气</t>
+        </is>
+      </c>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>每日顶空注入约2.08 L空气；1%储气袋体积</t>
+        </is>
+      </c>
+      <c r="R108" s="2" t="inlineStr">
+        <is>
+          <t>二重复微曝气储气袋与二重复氧化铁过滤</t>
+        </is>
+      </c>
       <c r="S108" s="2" t="inlineStr"/>
       <c r="T108" s="2" t="inlineStr"/>
       <c r="U108" s="2" t="inlineStr"/>
-      <c r="V108" s="2" t="inlineStr"/>
-      <c r="W108" s="2" t="inlineStr"/>
+      <c r="V108" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.5（PDF4–6页）为消化/微曝气/铁滤、SOB培养和Gram染色、气体/元素和统计；分离纯培养没有基因组或群落组学测序。</t>
+        </is>
+      </c>
+      <c r="W108" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–14页定位；方法PDF4–6页§2</t>
+        </is>
+      </c>
       <c r="X108" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05472/fulltext/fulltext__published__a81227cda8f65dc0.pdf"]</t>
@@ -14020,13 +14740,21 @@
       <c r="AB108" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC108" s="2" t="inlineStr"/>
+      <c r="AC108" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE108" s="2" t="inlineStr"/>
+          <t>["R05472-E01"]</t>
+        </is>
+      </c>
+      <c r="AE108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:14:31.726362+00:00</t>
+        </is>
+      </c>
       <c r="AF108" s="2" t="inlineStr"/>
     </row>
     <row r="109" ht="60" customHeight="1">
@@ -14177,22 +14905,62 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K110" s="2" t="inlineStr"/>
-      <c r="L110" s="2" t="inlineStr"/>
-      <c r="M110" s="2" t="inlineStr"/>
-      <c r="N110" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>16S扩增子MiSeq + PICRUSt功能预测（非目标）</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O110" s="2" t="inlineStr"/>
-      <c r="P110" s="2" t="inlineStr"/>
-      <c r="Q110" s="2" t="inlineStr"/>
-      <c r="R110" s="2" t="inlineStr"/>
-      <c r="S110" s="2" t="inlineStr"/>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>厕所黑水</t>
+        </is>
+      </c>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>0/5/10/50/150 mg O2/L反应器/周期</t>
+        </is>
+      </c>
+      <c r="R110" s="2" t="inlineStr">
+        <is>
+          <t>五个ASBR梯度氧，HRT5/4/3/2天</t>
+        </is>
+      </c>
+      <c r="S110" s="2" t="inlineStr">
+        <is>
+          <t>Illumina MiSeq（16S）</t>
+        </is>
+      </c>
       <c r="T110" s="2" t="inlineStr"/>
       <c r="U110" s="2" t="inlineStr"/>
-      <c r="V110" s="2" t="inlineStr"/>
-      <c r="W110" s="2" t="inlineStr"/>
+      <c r="V110" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.4（PDF2–3页）明确515F/806R扩增16S、MiSeq、QIIME2/DADA2，再用PICRUSt预测metagenome/functions；未实际shotgun/RNA测序。现有DOCX为黑水指标和pH/VFA/EEM图。</t>
+        </is>
+      </c>
+      <c r="W110" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–8页定位；方法PDF2–3页；预测说明PDF5–6页；DOCX全部42段落</t>
+        </is>
+      </c>
       <c r="X110" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05511/fulltext/fulltext__published__f020eb6189063184.pdf"]</t>
@@ -14216,13 +14984,21 @@
       <c r="AB110" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC110" s="2" t="inlineStr"/>
+      <c r="AC110" s="2" t="inlineStr">
+        <is>
+          <t>题名/作者匹配SI仅1表3图，无额外组学流程或编号。</t>
+        </is>
+      </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE110" s="2" t="inlineStr"/>
+          <t>["R05511-E01", "R05511-E02", "R05511-E03"]</t>
+        </is>
+      </c>
+      <c r="AE110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:14:31.762956+00:00</t>
+        </is>
+      </c>
       <c r="AF110" s="2" t="inlineStr"/>
     </row>
     <row r="111" ht="60" customHeight="1">
@@ -14273,22 +15049,54 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K111" s="2" t="inlineStr"/>
-      <c r="L111" s="2" t="inlineStr"/>
-      <c r="M111" s="2" t="inlineStr"/>
-      <c r="N111" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；流式细胞术、ATP及理化</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O111" s="2" t="inlineStr"/>
-      <c r="P111" s="2" t="inlineStr"/>
-      <c r="Q111" s="2" t="inlineStr"/>
+      <c r="P111" s="2" t="inlineStr">
+        <is>
+          <t>70%浓缩生物污泥+30%初沉污泥</t>
+        </is>
+      </c>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>0.1–0.5 vvm预曝气，优化0.2 vvm、40h</t>
+        </is>
+      </c>
       <c r="R111" s="2" t="inlineStr"/>
       <c r="S111" s="2" t="inlineStr"/>
       <c r="T111" s="2" t="inlineStr"/>
       <c r="U111" s="2" t="inlineStr"/>
-      <c r="V111" s="2" t="inlineStr"/>
-      <c r="W111" s="2" t="inlineStr"/>
+      <c r="V111" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.4.3（PDF2–4页）为预处理/AD反应器、Annexin/PI流式细胞生死染色、ATP发光及标准水质/GC，非宏转录组或宏基因组。</t>
+        </is>
+      </c>
+      <c r="W111" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–11页定位；方法PDF2–4页§2</t>
+        </is>
+      </c>
       <c r="X111" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05542/fulltext/fulltext__published__735560cdb2769e25.pdf"]</t>
@@ -14312,13 +15120,21 @@
       <c r="AB111" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC111" s="2" t="inlineStr"/>
+      <c r="AC111" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE111" s="2" t="inlineStr"/>
+          <t>["R05542-E01", "R05542-E02"]</t>
+        </is>
+      </c>
+      <c r="AE111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:14:31.795500+00:00</t>
+        </is>
+      </c>
       <c r="AF111" s="2" t="inlineStr"/>
     </row>
     <row r="112" ht="60" customHeight="1">
@@ -14369,22 +15185,54 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K112" s="2" t="inlineStr"/>
-      <c r="L112" s="2" t="inlineStr"/>
-      <c r="M112" s="2" t="inlineStr"/>
-      <c r="N112" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；产气、水质和数学模型</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O112" s="2" t="inlineStr"/>
-      <c r="P112" s="2" t="inlineStr"/>
-      <c r="Q112" s="2" t="inlineStr"/>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>餐厨废物</t>
+        </is>
+      </c>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>0/5/10/15/20 mL氧</t>
+        </is>
+      </c>
       <c r="R112" s="2" t="inlineStr"/>
       <c r="S112" s="2" t="inlineStr"/>
       <c r="T112" s="2" t="inlineStr"/>
       <c r="U112" s="2" t="inlineStr"/>
-      <c r="V112" s="2" t="inlineStr"/>
-      <c r="W112" s="2" t="inlineStr"/>
+      <c r="V112" s="2" t="inlineStr">
+        <is>
+          <t>完整Materials and methods（PDF2页）及Table2（PDF3页）为SBR发酵、产气、pH、COD、氨氮；sequencing batch指序批反应器，不是测序。未报告组学。</t>
+        </is>
+      </c>
+      <c r="W112" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–7页定位；方法PDF2页；Table2 PDF3页</t>
+        </is>
+      </c>
       <c r="X112" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05543/fulltext/fulltext__published__b9b6c6f484001832.pdf"]</t>
@@ -14408,13 +15256,21 @@
       <c r="AB112" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC112" s="2" t="inlineStr"/>
+      <c r="AC112" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE112" s="2" t="inlineStr"/>
+          <t>["R05543-E01"]</t>
+        </is>
+      </c>
+      <c r="AE112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:14:31.837445+00:00</t>
+        </is>
+      </c>
       <c r="AF112" s="2" t="inlineStr"/>
     </row>
     <row r="113" ht="60" customHeight="1">
@@ -14465,22 +15321,58 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="K113" s="2" t="inlineStr"/>
-      <c r="L113" s="2" t="inlineStr"/>
-      <c r="M113" s="2" t="inlineStr"/>
-      <c r="N113" s="2" t="inlineStr"/>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>未使用目标测序</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>未报告测序；消化稳定性及理化分析</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>不适用（未使用目标测序）</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
       <c r="O113" s="2" t="inlineStr"/>
-      <c r="P113" s="2" t="inlineStr"/>
-      <c r="Q113" s="2" t="inlineStr"/>
-      <c r="R113" s="2" t="inlineStr"/>
+      <c r="P113" s="2" t="inlineStr">
+        <is>
+          <t>猪粪高固体AD</t>
+        </is>
+      </c>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>本研究纳米气泡水为CO2制备（原范围分类保留）</t>
+        </is>
+      </c>
+      <c r="R113" s="2" t="inlineStr">
+        <is>
+          <t>3/6/8/10%TS，NBW与去离子水对照</t>
+        </is>
+      </c>
       <c r="S113" s="2" t="inlineStr"/>
       <c r="T113" s="2" t="inlineStr"/>
       <c r="U113" s="2" t="inlineStr"/>
-      <c r="V113" s="2" t="inlineStr"/>
-      <c r="W113" s="2" t="inlineStr"/>
+      <c r="V113" s="2" t="inlineStr">
+        <is>
+          <t>完整§2.1–2.4（PDF2–3页）为批次AD、CO2纳米气泡水、产气/固体/碱度/氨/VFA/蛋白糖和统计，无DNA/RNA建库或测序。不因气体为CO2改原研究范围。</t>
+        </is>
+      </c>
+      <c r="W113" s="2" t="inlineStr">
+        <is>
+          <t>全文PDF1–9页定位；方法PDF2–3页§2</t>
+        </is>
+      </c>
       <c r="X113" s="2" t="inlineStr">
         <is>
           <t>["original_files/R05544/fulltext/fulltext__published__24c76324a7cd3191.pdf"]</t>
@@ -14504,13 +15396,21 @@
       <c r="AB113" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AC113" s="2" t="inlineStr"/>
+      <c r="AC113" s="2" t="inlineStr">
+        <is>
+          <t>当前无独立补充原件；不据此认定不存在SI。</t>
+        </is>
+      </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AE113" s="2" t="inlineStr"/>
+          <t>["R05544-E01", "R05544-E02"]</t>
+        </is>
+      </c>
+      <c r="AE113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T09:14:50.414176+00:00</t>
+        </is>
+      </c>
       <c r="AF113" s="2" t="inlineStr"/>
     </row>
     <row r="114" ht="60" customHeight="1">
@@ -45329,7 +46229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L158"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -54080,8 +54980,2259 @@
         </is>
       </c>
     </row>
+    <row r="159" ht="90" customHeight="1">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>R04646-E01</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>R04646</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Samples
+ taken
+ from
+ the
+ outlet
+ of
+ the
+ reactors
+ at
+ the
+ end
+ of
+the
+ cycle
+ time
+ were
+ analyzed
+ three
+ times
+ a
+ week
+ by
+ measuring
+pH,
+ alkalinity,
+ oxidation-reduction
+ potential
+ (ORP),
+ dissolved
+oxygen
+ (DO),
+ salinity,
+ COD,
+ DB22
+ concentration,
+ and
+ aromatic
+amines
+ (qualitatively).</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>完整方法为水质、染料/芳香胺光谱及GC，无目标测序。</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04646/fulltext/fulltext__published__e1d4e0f3c97d519f.pdf</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>e1d4e0f3c97d519f1a419d98a6493eec88f5ce98834b86c2c0831c2c96908766</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>2.3 Analytical procedure</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr"/>
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="90" customHeight="1">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>R04646-E02</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>R04646</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Acute
+ ecotoxicity
+ of
+ the
+ inﬂuent
+ and
+ efﬂuent
+ of
+ each
+ reac-
+tor
+ was evaluated
+ at
+ the
+ end
+ of
+ the
+ operational
+ period
+ by
+Microtox® (Microtox
+ Model
+ 500
+ analyzer,
+ Strategic
+ Diagnos-
+tics,
+ Inc.
+ SDIX,
+ Newark,
+ DE,
+ USA),
+ applying
+ the
+ bioluminescent
+bacterium
+ Vibrio
+ ﬁscheri
+ as
+ the
+ toxicity
+ indicator
+ (incubation
+time
+ of
+ 15
+ min).</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Microtox为生物发光毒性试验，不是组学测序。</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04646/fulltext/fulltext__published__e1d4e0f3c97d519f.pdf</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>e1d4e0f3c97d519f1a419d98a6493eec88f5ce98834b86c2c0831c2c96908766</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>2.3 Analytical procedure</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr"/>
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="90" customHeight="1">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>R04700-E01</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>R04700</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>Next, bio-methane potential (BMP) test, gas chromatography (GC)
+and particle size distribution analysis were carried out to estimate the methane potential
+and biogas composition of the aerated and non-aerated sludge.</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>完整方法为BMP、GC与粒径分析，无核酸/建库流程。</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04700/fulltext/fulltext__thesis__40ac0de29f75851c.pdf</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>40ac0de29f75851cab1651e1e339d03329bb7ce0141519329487f0559ebd8297</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>[14]</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>3 Materials and Methodology</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr"/>
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="90" customHeight="1">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>R04700-E02</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>R04700</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>The 0 bar, 5 bar aerated and 5 bar supernatant samples were tested to analyze the effect
+of aeration on particle size distribution. The Bluewave – Particle Size Analyzer (PSA) from
+Microtrac was used for this analysis. The procedure followed was based on the Bulewave
+particle size analyzer user manual (Microtrac, 2019).</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>粒径检测仪器，不是微生物组测序。</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04700/fulltext/fulltext__thesis__40ac0de29f75851c.pdf</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>40ac0de29f75851cab1651e1e339d03329bb7ce0141519329487f0559ebd8297</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>[22]</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>3.5 Particle Size Distribution</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr"/>
+      <c r="L162" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="90" customHeight="1">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>R04786-E01</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>R04786</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA genes fragments were
+ampliﬁed from the obtained DNA using a primer set, 338F (5′-ACTCC
+TACGGGAGGCAGCAG-3′)
+and
+806R
+(5-’GGACTACHVGGGTWTCT-
+AAT-3′) for bacteria, and Arch524F (5-’TG YCAGCCGCCGCGGTAA-3′)
+and Arch958R (5-′YCCGGCGTTGAVTCCAATT-3′) for archaea. Puriﬁed
+amplicons were pooled in equimolar, and paired-end sequenced on an
+Illumina-MiSeq platform. Then 16S rRNA sequences were clustered into
+operational taxonomic units by setting a 3% distance limit.</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>靶基因/引物与amplicon池化明确，非宏基因组。</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04786/fulltext/fulltext__published__ea18005b6cd10f40.pdf</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>ea18005b6cd10f402de201443be02098d554b7564b6d6aa3cf6713b5c861946c</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>2.4.1 Bacterial and archaeal community</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr"/>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="90" customHeight="1">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>R04796-E01</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>R04796</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Untreated and treated biogas were analyzed to detect daily and
+seasonal diﬀerences using two portable continuous biogas testing and monitoring systems (Siemens
+Model #7MB2337-3CR13-5DR1, Siemens AG, Munich, Germany) for CH4 (0% to 100%), CO2 (0%
+to 100%), O2 (0% to 100%), and H2S (0–5000 ppm), with a Campbell Scientiﬁc CR1000 data logger
+and acquisition system, and gas meters (Model #9500, Thermal Instrument Co, Trevose, PA, USA;
+Model #FT2, Fox Thermal, Marina, CA, USA) and assembled as described in Shelford et al. 2019 [4].</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>测量为CH4/CO2/O2/H2S传感及气量，无目标测序。</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04796/fulltext/fulltext__published__6844f12fe56c174d.pdf</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>6844f12fe56c174d2250e0a88bba570a3c94fd37dec91d66d805c2cec1c2c013</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>2.2 Performance Monitoring and Cost Information</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr"/>
+      <c r="L164" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="90" customHeight="1">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>R04803-E01</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>R04803</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Bacterial and archaeal community structure was analyzed by PCR-
+DGGE (Ploymerase Chain Reaction Denaturing Gradient Gel Electrophoresis) 
+according to [9]. The obtained archaeal and bacterial DGGE gels were analyzed in order 
+to calculate the following ecological parameters: evenness/functional organization (Fo), 
+ranged weighted richness (Rr) and Shannon diversity index (H) according to [22].</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>微生物结构采用PCR-DGGE及其指纹指数，不是宏基因组/宏转录组。</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04803/fulltext/fulltext__published__3e98d6cf0fefd5e7.pdf</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>3e98d6cf0fefd5e7daae2600b11ecc00cdff35ca4f4dfd462e4c7ed25bb3c6c6</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>[6]</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>2.5 Analytical methods</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr"/>
+      <c r="K165" s="2" t="inlineStr"/>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="90" customHeight="1">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>R04889-E01</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>R04889</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Measured variables reported in this 
+study included pH, sCOD, volatile fatty acid 
+(VFA), methane production, and anaerobic total 
+plate count.</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>菌量以培养平板计数，非宏基因组/宏转录组。</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04889/fulltext/fulltext__published__860a0532503787f8.pdf</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>860a0532503787f8bb84a599bdbf923f690615b05121c8a78c21249f8de911cb</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>RESEARCH METHODOLOGY – Anaerobic digestion</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr"/>
+      <c r="K166" s="2" t="inlineStr"/>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="90" customHeight="1">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>R04889-E02</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>R04889</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>Analysis of sCOD and VFA were 
+conducted 
+by 
+following 
+APHA 
+procedures 
+(Clesceri, et.al., 2005). Methane concentration was 
+measured using Gas Chromatography Shimadzu 
+GC 8A.</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>完整检测为水质、VFA和产气GC。</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04889/fulltext/fulltext__published__860a0532503787f8.pdf</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>860a0532503787f8bb84a599bdbf923f690615b05121c8a78c21249f8de911cb</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>RESEARCH METHODOLOGY – Analysis</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr"/>
+      <c r="K167" s="2" t="inlineStr"/>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="90" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>R04899-E01</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>R04899</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>The bacterial and methanogenic communities were investigated
+by targeting the 16S rRNA gene using 515F/806R primers and the
+mcrA gene using mcrA3F/mcrA3R primers, respectively (Caporaso
+et al., 2012; Luton et al., 2002).</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>靶标为16S及mcrA，非群落DNA随机建库。</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04899/fulltext/fulltext__published__92f0b2f1ad01522c.pdf</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>92f0b2f1ad01522ccc4e76595e3cd022e18db61eb7367bec31eeb097881b8329</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>2.5 Microbial analyses</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr"/>
+      <c r="K168" s="2" t="inlineStr"/>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="90" customHeight="1">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>R04899-E02</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>R04899</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>非目标编号排除</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>The raw sequence reads were
+deposited in the NCBI Sequence Read Archive (SRA; http://www.
+ncbi.nlm.nih.gov/sra) under accession numbers SAMN12752316 to
+SAMN12752321 and SAMN12752323 to SAMN12752328.</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>文中给出BioSample编号，属于上述标记基因数据，不计为目标组学项目。</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04899/fulltext/fulltext__published__92f0b2f1ad01522c.pdf</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>92f0b2f1ad01522ccc4e76595e3cd022e18db61eb7367bec31eeb097881b8329</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>2.5 Microbial analyses</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr"/>
+      <c r="K169" s="2" t="inlineStr"/>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="90" customHeight="1">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>R04899-E03</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>R04899</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>术语命中排除</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>How-
+ever, further metatranscriptomic analyses are needed to evaluate</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>明确未来需要宏转录组，不能视作实际开展。</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04899/fulltext/fulltext__published__92f0b2f1ad01522c.pdf</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>92f0b2f1ad01522ccc4e76595e3cd022e18db61eb7367bec31eeb097881b8329</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>[7]</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>4 Discussion</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr"/>
+      <c r="K170" s="2" t="inlineStr"/>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="90" customHeight="1">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>R04899-E04</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>R04899</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting materials and methods: </t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>补充方法列表为ORP/化学/热力学，现有附件无额外目标测序流程。</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04899/supplementary/supplementary__93e7e6da6f9fc16c.docx</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>93e7e6da6f9fc16c9535a4cfd721b7da589326e3314fb7eee286572c71da81eb</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>DOCX段落20–23、40–80；Table S2段落109–377</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr"/>
+      <c r="K171" s="2" t="inlineStr"/>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="90" customHeight="1">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>R04912-E01</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>R04912</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Five parallel groups were 
+set up. Group 1 was used as a control and it was carried out as a standard anaerobic 
+fermentation. Groups 2–5 were experimental groups, and 5 ml, 10 ml, 15 ml, and 20 ml 
+of air were respectively inflated to create different microaerobic conditions. The biogas 
+generation in each group was measured once a day, and the total amount of biogas 
+generation in each group was also calculated.</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>实验测量每日沼气体积，非测序；微生物生长模型不等同组学。</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04912/fulltext/fulltext__published__ba09ba8854601318.pdf</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>ba09ba8854601318e3af61c59c8980e8022ec2a668e0c1f925cc16502a53081b</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>Experimental methods</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr"/>
+      <c r="K172" s="2" t="inlineStr"/>
+      <c r="L172" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="90" customHeight="1">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>R04922-E01</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>R04922</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Biogas composition (CH4, CO2,
+H2S and O2) in the three digesters and upstream of the CHP unit was
+monitored six times/day using an Optima 7 portable biogas analyzer
+(MRU GmbH, Germany).</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>测量气体组分，完整方法无目标测序。</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04922/fulltext/fulltext__published__d4f609c42961a5d2.pdf</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>d4f609c42961a5d25218af73e99fcc5ae1f02a5018337ec964fe076fc1addcbf</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>2.3 Monitoring and analytical methods</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr"/>
+      <c r="K173" s="2" t="inlineStr"/>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="90" customHeight="1">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>R04928-E01</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>R04928</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Once daily, 300 ml samples were taken for VS and 
+VFA analysis through sampling valve. The VS and VFA 
+analysis was done in 3 series per day per digester and 
+followed by APHA (American Public Health Association - 
+APHA, 2005).</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>检测VS/VFA及沼气体积，无目标测序。</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04928/fulltext/fulltext__published__9d47028c02204ac0.pdf</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>9d47028c02204ac08f73849bdf73af55c1e235aa3593b2b281d139b85d58607f</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>2.2 Experimental</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr"/>
+      <c r="K174" s="2" t="inlineStr"/>
+      <c r="L174" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="90" customHeight="1">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>R05065-E01</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>R05065</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>The V3-V4 regions of the 16 s rDNA genes were am-
+plified with 340 F (CCTACGGGNBGCASCAG) and 805R (GACTACNV-
+GGGTATCTAATCC). All polymerase chain reaction (PCR) reaction
+mixture was purified with the MinElute Gel Extraction Kit (Qiagen,
+Germany). The Invitrogen™-Qubit fluorometer quantitative system
+(California, USA) was used to quantity the amplicons. Then high-
+throughput sequencing of 16S DNA amplicons were sequenced with the
+Illumina MiSeq platform at SinoGenoMax Co., Ltd (Beijing, China).</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>明确扩增16S并测amplicons，非宏基因组。</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05065/fulltext/fulltext__published__239adeaf9a5df55a.pdf</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>239adeaf9a5df55a383ba454cf2811563b710d89e446a0af02062140664e382e</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>2.6 Microbial structure analysis</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr"/>
+      <c r="K175" s="2" t="inlineStr"/>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="90" customHeight="1">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>R05065-E02</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>R05065</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Table S2 Community richness and diversity indices of different samples</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>补充表是16S群落丰富度/多样性，不是shotgun库。</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05065/supplementary/supplementary__138834a73b710b94.docx</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>138834a73b710b94f194521b56815619a34161b6ccdb225f771fb58e8ede57bb</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>DOCX Table S2，段落290–346</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr"/>
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="90" customHeight="1">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>R05173-E01</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>R05173</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA
+genes were ampliﬁed using the bacterial universal primers (515F
+and 806R) with speciﬁc barcode.</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>靶基因引物明确，非shotgun。</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05173/fulltext/fulltext__published__dedf2d646e952ba0.pdf</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>dedf2d646e952ba0f6c2e7326d6c8ceda5eac7f0c9485dba3a4a0d136a922526</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA amplicon sequencing and data processing</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr"/>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="90" customHeight="1">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>R05173-E02</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>R05173</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>PCR products were quantiﬁed, mixed, puriﬁed and
+sequenced on an Illumina HiSeq platform at Novogene (Beijing,
+China).</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>HiSeq用于PCR产物，不按平台判断宏基因组。</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05173/fulltext/fulltext__published__dedf2d646e952ba0.pdf</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>dedf2d646e952ba0f6c2e7326d6c8ceda5eac7f0c9485dba3a4a0d136a922526</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>16S rRNA amplicon sequencing and data processing</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr"/>
+      <c r="K178" s="2" t="inlineStr"/>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="90" customHeight="1">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>R05173-E03</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>R05173</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Physicochemical characteristics of seed sludge.</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>仅种泥理化表及相关图；保持唯一归属待核实。</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05173/supplementary/supplementary__63ce6947f3cf6519.docx</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>63ce6947f3cf65197f9c19d5a0ba14d1e8d45197745c67215e1350d8d6b586e6</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>DOCX段落1–23、41–45</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr"/>
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="90" customHeight="1">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>R05213-E01</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>An LPMO from 
+Neurospora crassa (NcLPMO9C) was expressed and 
+purified as described by Müller et al. [21].</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>蛋白酶制剂表达纯化不构成宏转录组。</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05213/fulltext/fulltext__published__bcab84a15ce93062.pdf</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>[11]</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>Methods – Enzyme preparations</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr"/>
+      <c r="K180" s="2" t="inlineStr"/>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="90" customHeight="1">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>R05213-E02</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>The biogas composition 
+was assessed using a gas chromatograph (3000 Micro 
+GC, Agilent Technologies, USA) equipped with a ther-
+mal conductivity detector (TCD), allowing detection of 
+methane, carbon-dioxide and nitrogen gas.</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>完整方法为酶/产物与产气分析，无目标测序。</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05213/fulltext/fulltext__published__bcab84a15ce93062.pdf</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>[12]</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>Methods – Biogas analysis and calculation</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr"/>
+      <c r="K181" s="2" t="inlineStr"/>
+      <c r="L181" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="90" customHeight="1">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>R05213-E03</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>非目标泛指索取声明</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Additional data are available from the corresponding author on reasonable 
+request.</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>泛指研究数据，不是相关原始测序数据声明；无目标测序，不计可索取命中。</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05213/fulltext/fulltext__published__bcab84a15ce93062.pdf</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>[13]</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>Availability of data and materials</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr"/>
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="90" customHeight="1">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>R05213-E04</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Figure S1. (A) Chromatogram of soluble fractions of anaerobic digestion reactions with Avicel supplemented with purified NcLPMO9C as well as H2O2. Samples were taken initially in reactions supplemented with purified NcLPMO9C, after addition of H2O2 or H2O. Shoulder peaks representing Glc4gemGlc, seen in reactions with NcLPMO9C only, are highlighted by the dashed lines. (B) Chromatogram of a standard sample (0,001 g/L) obtained after treating cellopentaose with NcLPMO9C, run together with other samples.</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>色谱及甲烷曲线，未包含测序方法或编号。</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05213/supplementary/supplementary__2a8184a309e33621.docx</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>2a8184a309e3362192b49457a6cae5f0da5f682d39e48fee2b3dcbfc67a87853</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>DOCX Figure S1–S7，段落23–71</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr"/>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="90" customHeight="1">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>R05319-E01</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>R05319</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Forward primers
+(338F and 524F) and reverse primers (806R and 958R) for bacterial
+and archaeal sequences, respectively, were performed for ampliﬁca-
+tions of 16S rDNA. The key characteristics of PCR thermal cycling
+were taken from a previous study.3 PCR products were then puriﬁed,
+quantitated, and paired-end-sequenced based on the platform of
+Illumina MiSeq</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>16S靶基因扩增及PCR产物测序，非宏基因组。</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05319/fulltext/fulltext__published__865dcb7f90757119.pdf</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>865dcb7f90757119fcc3c78c4e24b37817c7bf203a8727ab8e54a7d37304e19c</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>2.5 Microbial Community Analysis</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr"/>
+      <c r="K184" s="2" t="inlineStr"/>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="90" customHeight="1">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>R05319-E02</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>R05319</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>术语命中排除</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>The complete genome sequence for putative H2- and S-oxidizer
+candidatus Sulfuricurvum sp. assembled de novo from an aquifer-
+derived metagenome.</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>被引论文题名，不是本研究测序或公开数据复用。</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05319/fulltext/fulltext__published__865dcb7f90757119.pdf</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>865dcb7f90757119fcc3c78c4e24b37817c7bf203a8727ab8e54a7d37304e19c</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>References (43)</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
+      <c r="K185" s="2" t="inlineStr"/>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="90" customHeight="1">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>R05396-E01</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>R05396</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>The microbial community structure analysis of pretreatment liquid
+showed that there were a total of 16 identified bacterial phyla and a
+total of 7 identified fungal class. The most dominant bacterial phyla was
+Bacteroidetes (50.26%), and followed by Firmicutes (15.37%) and Pro-
+teobacteria (9.34%). The most dominant fungal class was Sordar-
+iomycetes (44.99%), and followed by Dothideomycetes (25.56%) and
+Eurotiomycetes (17.9%).</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>报告群落组成但未说明分析方法，不能推断目标或非目标测序。</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05396/fulltext/fulltext__published__0a746b3ef69be3a5.pdf</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>0a746b3ef69be3a5b775f72e10dc44c95fe93c381373a8c5ecae4eb65f83a4f5</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>2.1 Raw materials</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr"/>
+      <c r="K186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="90" customHeight="1">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>R05396-E02</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>R05396</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Fig. A.1 Mycelium morphology of ORS surface in different pretreatment time.</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>现有附件为菌丝形态/显微与材料结构图，无核酸/建库证据。</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05396/supplementary/supplementary__5e7c6f02f21c479f.docx</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>5e7c6f02f21c479f48987d2f27f3c857f5a7f2605b6728de78ced29d7358a0be</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>DOCX段落14、17、19、21</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr"/>
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="90" customHeight="1">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>R05472-E01</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>R05472</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>The criteria for identifying SOB-positive tubes
+were (1) visualization of the turbidity of the medium, (2) microscopic veriﬁcation of the growth of
+the microorganism in the medium liquid using an optical microscope, and (3) observation of the
+presence of colonies in the solids.</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>SOB鉴定为培养浊度、显微与菌落，不是序列测定。</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05472/fulltext/fulltext__published__a81227cda8f65dc0.pdf</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>a81227cda8f65dc0a1784d367c05e5848d87660afd9c7b9c1cb20770f1aa37b0</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>[5]</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>2.3 Sulfur-Oxidizing Bacteria Observation and Isolation</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
+      <c r="K188" s="2" t="inlineStr"/>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="90" customHeight="1">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>R05511-E01</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>R05511</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>PCR was performed followed by
+sequencing on the Illumina MiSeq platform. The 16S rRNA genes
+were
+ampliﬁed
+using
+the
+universal
+primer
+pair
+515F
+(GTGCCAGCMGCCGCGG) and 806R (GGACTACHVGGGTWTCTAAT).</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>16S靶基因扩增，不是群落DNA随机测序。</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05511/fulltext/fulltext__published__f020eb6189063184.pdf</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>f020eb6189063184de1d86419290cfe595da970bbf395020168c0ce5a8349e91</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>2.4 Microbial analysis</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr"/>
+      <c r="K189" s="2" t="inlineStr"/>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="90" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>R05511-E02</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>R05511</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>功能预测排除</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>The predicted metagenome and
+functional genes were determined using the Phylogenetic Investi-
+gation of Communities by Reconstruction of Unobserved States
+(PICRUSt) (Langille et al., 2013).</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>明确PICRUSt预测，不能计为实际宏基因组。</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05511/fulltext/fulltext__published__f020eb6189063184.pdf</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>f020eb6189063184de1d86419290cfe595da970bbf395020168c0ce5a8349e91</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>2.4 Microbial analysis</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr"/>
+      <c r="K190" s="2" t="inlineStr"/>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="90" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>R05511-E03</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>R05511</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>补充材料核查</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Table S1. Characterization of conventional flush toilets blackwater</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>现有补充仅水质表与pH/VFA/EEM图，无额外目标测序。</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05511/supplementary/supplementary__b434b7fc5acd7ee0.docx</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>b434b7fc5acd7ee0b4792e0ca5a2017a4ed1991e88eee3baf94c1bfcde86721b</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>DOCX段落8–10、14–41</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr"/>
+      <c r="K191" s="2" t="inlineStr"/>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="90" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>R05542-E01</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>R05542</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>To this end, the apoptosis
+evaluation kit containing specic Annexin and propidium
+iodide were used.</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>流式细胞荧光染色，不是测序。</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05542/fulltext/fulltext__published__735560cdb2769e25.pdf</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>735560cdb2769e2517355c073dd51a95ac90b015a5b36f90dcc0dff360ae182b</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>2.4.1 Flow cytometry assay</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr"/>
+      <c r="K192" s="2" t="inlineStr"/>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="90" customHeight="1">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>R05542-E02</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>R05542</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>ATP biolog-
+ical measurement was performed to determine the quantify
+the metabolic activity in the biological medium using the ATP
+kit (AquaSnap™Total (Hygiena)).</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>ATP为生化发光测量，不是RNA测序。</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05542/fulltext/fulltext__published__735560cdb2769e25.pdf</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>735560cdb2769e2517355c073dd51a95ac90b015a5b36f90dcc0dff360ae182b</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>2.4.2 ATP measurement</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr"/>
+      <c r="L193" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="90" customHeight="1">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>R05543-E01</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>R05543</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>The variation patterns of primary parameters such as 
+daily gas production, cumulative gas production, pH, COD, 
+and ammonia nitrogen were evaluated. The detection meth-
+ods, instrument models, and measurement accuracy of these 
+parameters are shown in Table 2.</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>检测指标为产气/pH/COD/氨氮，表2仪器亦为水质与气体仪，无测序。</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05543/fulltext/fulltext__published__b9b6c6f484001832.pdf</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>b9b6c6f4840018324ed13892f9b0e35390e8ddbad76f3aab938611304261daed</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>Experimental methods</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr"/>
+      <c r="K194" s="2" t="inlineStr"/>
+      <c r="L194" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="90" customHeight="1">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>R05544-E01</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>R05544</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>In-
+troduced carbon dioxide gas into deionized water (DW) through this
+generator at 20 ± 2 °C for 20 min to get NBW used throughout the AD
+process in this research.</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>气泡气体明示CO2；保持原分类，仅记录方法。</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05544/fulltext/fulltext__published__24c76324a7cd3191.pdf</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>24c76324a7cd319136713fab50e62f23646cac5f5f6a8abb0a4ca9560a4173f8</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>2.2 Preparation of NBW</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
+      <c r="K195" s="2" t="inlineStr"/>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="90" customHeight="1">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>R05544-E02</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>R05544</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>方法判断</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Soluble carbohydrates and proteins were determined by
+using the phenol–sulfuric method and Lowry method, respectively.</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>理化/比色及GC方法，无目标测序。</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05544/fulltext/fulltext__published__24c76324a7cd3191.pdf</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>24c76324a7cd319136713fab50e62f23646cac5f5f6a8abb0a4ca9560a4173f8</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>2.3 Analytical methods</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr"/>
+      <c r="K196" s="2" t="inlineStr"/>
+      <c r="L196" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L158"/>
+  <autoFilter ref="A1:L196"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -54092,7 +57243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -58521,8 +61672,158 @@
       <c r="O106" s="2" t="inlineStr"/>
       <c r="P106" s="2" t="inlineStr"/>
     </row>
+    <row r="107" ht="60" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>R04646</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>正文提及SI但当前无原件</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04646/fulltext/fulltext__published__e1d4e0f3c97d519f.pdf</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>e1d4e0f3c97d519f1a419d98a6493eec88f5ce98834b86c2c0831c2c96908766</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr"/>
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>§2.1/2.4称SI含染料NMR纯度及动力学计算，现无原件。</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>保留缺口；正文方法无目标测序，不追下载。</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr"/>
+      <c r="N107" s="2" t="inlineStr"/>
+      <c r="O107" s="2" t="inlineStr"/>
+      <c r="P107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108" ht="60" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>R04899</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>非目标扩增子BioSample编号</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R04899/fulltext/fulltext__published__92f0b2f1ad01522c.pdf</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>92f0b2f1ad01522ccc4e76595e3cd022e18db61eb7367bec31eeb097881b8329</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>SAMN12752316 to SAMN12752321 and SAMN12752323 to SAMN12752328</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>SAMN12752316–SAMN12752321; SAMN12752323–SAMN12752328</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>BioSample样本（非项目）</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>NCBI BioSample/SRA</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/biosample/?term=SAMN12752316</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>正文§2.5对应16S及mcrA扩增子，不是宏基因组/宏转录组；未逐个官方核验，也未将12个编号计为12项目。</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>保留非目标线索，不计目标项目。</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr"/>
+      <c r="N108" s="2" t="inlineStr"/>
+      <c r="O108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109" ht="60" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>R05396</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>测序类型待确认</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>original_files/R05396/fulltext/fulltext__published__0a746b3ef69be3a5.pdf</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>0a746b3ef69be3a5b775f72e10dc44c95fe93c381373a8c5ecae4eb65f83a4f5</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr"/>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>菌群组成已报告但核酸/测序方法及数据来源缺失；现有正文/匹配SI无法区分目标组学和标记基因。</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>独立复核队列；需要菌群分析的靶标/建库说明，不计阳性或阴性。</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr"/>
+      <c r="N109" s="2" t="inlineStr"/>
+      <c r="O109" s="2" t="inlineStr"/>
+      <c r="P109" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P106"/>
+  <autoFilter ref="A1:P109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -58533,7 +61834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -58619,7 +61920,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -58635,7 +61936,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -58767,7 +62068,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -58783,7 +62084,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -58848,7 +62149,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>R04646</t>
+          <t>R05550</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -59746,8 +63047,226 @@
       </c>
       <c r="D72" s="2" t="inlineStr"/>
     </row>
+    <row r="73" ht="60" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>本批完成ID</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>R04646, R04700, R04786, R04796, R04803, R04889, R04899, R04912, R04922, R04928, R05065, R05173, R05213, R05319, R05472, R05511, R05542, R05543, R05544</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>按稳定ID顺序，逐篇阅读方法；扫描件按需OCR/原页核查。 未解决项保留待确认，未标记完成或阴性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="60" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>research_screened_count</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75" ht="60" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>completed_count</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76" ht="60" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>pending_count</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77" ht="60" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>pending_ids</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>["R05396"]</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78" ht="60" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>processed_record_count</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>review_not_applicable_ids</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>target_articles</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>metagenomics_only</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82" ht="60" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>metatranscriptomics_only</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84" ht="60" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>public_data_articles</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85" ht="60" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>explicit_request_articles</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D72"/>
+  <autoFilter ref="A1:D85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>